<commit_message>
Catalogue: new items, video/title fixes, no bottom frame on mobile
- Add many new catalogue items (webp @1400px + thumbnails) and replace a few
  placeholder sets with full photo sets; all aligned to list.xlsx.
- Homepage hero: defer the video past first paint (poster shows immediately),
  so the initial load is no longer blocked by it on mobile.
- Fix the tab-title flash on the homepage (title now matches the template).
- Remove the bottom beige frame on mobile (its visualViewport pinning caused
  jumps); story text two points smaller on mobile.
- Catalogue hover: drop async decode on the hover image (was flashing white).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/list.xlsx
+++ b/src/assets/list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berna\OneDrive\Ambiente de Trabalho\FREELANCE\CONCEIÇÃO\WEBSITE CONCEIÇÃO\catalogue\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0370B3B8-013C-4FF3-8C65-9C136056CDDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CA5B45-5F01-447D-8A79-B6B5B186EEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="213">
   <si>
     <t>PRIORIDADE</t>
   </si>
@@ -891,90 +891,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="6" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1780,6 +1710,9 @@
       <c r="D30" s="10" t="s">
         <v>3</v>
       </c>
+      <c r="E30" s="18" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="31" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
@@ -3077,6 +3010,9 @@
       <c r="D123" s="10" t="s">
         <v>3</v>
       </c>
+      <c r="E123" s="18" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="124" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="s">
@@ -3152,6 +3088,9 @@
       </c>
       <c r="D128" s="10" t="s">
         <v>3</v>
+      </c>
+      <c r="E128" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="129" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3313,19 +3252,19 @@
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="A2:D139">
-    <cfRule type="expression" dxfId="19" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$D2="Alta"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
       <formula>$D2="Média"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$D2="Baixa"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
       <formula>$D2="Vendida"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
       <formula>$D2="Nula"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>